<commit_message>
Excel Update 18 Shahrivar
</commit_message>
<xml_diff>
--- a/Campaigns_Master.xlsx
+++ b/Campaigns_Master.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Good KoDz\Banner Monitor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0483A63F-1C18-47B9-95A4-B820A828B9BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4CE86CC-04F4-4110-A083-6F72CFC43DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EBB7D5F9-BF11-4273-8F7B-7CCC7D024DDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1326" uniqueCount="984">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1343" uniqueCount="984">
   <si>
     <t>Campaign Name</t>
   </si>
@@ -3322,7 +3325,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -3345,12 +3348,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -3406,6 +3420,7 @@
     <xf numFmtId="0" fontId="0" fillId="49" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="50" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3422,6 +3437,798 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Sheet1"/>
+      <sheetName val="Sheet2"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1">
+        <row r="1">
+          <cell r="A1" t="str">
+            <v>Campaign Name</v>
+          </cell>
+          <cell r="B1" t="str">
+            <v>Account Manager</v>
+          </cell>
+          <cell r="C1" t="str">
+            <v>Start Date</v>
+          </cell>
+          <cell r="D1" t="str">
+            <v>End Date</v>
+          </cell>
+          <cell r="E1" t="str">
+            <v>Price</v>
+          </cell>
+        </row>
+        <row r="2">
+          <cell r="A2" t="str">
+            <v>Dr Amir Azizi</v>
+          </cell>
+          <cell r="B2" t="str">
+            <v>Sanam</v>
+          </cell>
+          <cell r="C2" t="str">
+            <v>1405/04/06</v>
+          </cell>
+          <cell r="D2" t="str">
+            <v>1405/07/06</v>
+          </cell>
+          <cell r="E2">
+            <v>30600000</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="A3" t="str">
+            <v>DR Ali Saeedi</v>
+          </cell>
+          <cell r="B3" t="str">
+            <v>shahrzad</v>
+          </cell>
+          <cell r="C3" t="str">
+            <v>1405/03/26</v>
+          </cell>
+          <cell r="D3" t="str">
+            <v>1405/06/25</v>
+          </cell>
+          <cell r="E3">
+            <v>55000000</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="A4" t="str">
+            <v>DR Ali NaserBakhT</v>
+          </cell>
+          <cell r="B4" t="str">
+            <v>elahe</v>
+          </cell>
+          <cell r="C4" t="str">
+            <v>1405/02/29</v>
+          </cell>
+          <cell r="D4" t="str">
+            <v>1405/05/29</v>
+          </cell>
+          <cell r="E4">
+            <v>132000000</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="A5" t="str">
+            <v>Dr AssaEi</v>
+          </cell>
+          <cell r="B5" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C5" t="str">
+            <v>1405/05/26</v>
+          </cell>
+          <cell r="D5" t="str">
+            <v>1405/08/26</v>
+          </cell>
+          <cell r="E5">
+            <v>20000000</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="A6" t="str">
+            <v>DR Azadeh Khalajian</v>
+          </cell>
+          <cell r="B6" t="str">
+            <v>Sanam</v>
+          </cell>
+          <cell r="C6" t="str">
+            <v>1405/03/15</v>
+          </cell>
+          <cell r="D6" t="str">
+            <v>1405/06/15</v>
+          </cell>
+          <cell r="E6">
+            <v>60000000</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="A7" t="str">
+            <v>Dr Atefe Faramarzi</v>
+          </cell>
+          <cell r="B7" t="str">
+            <v>Naser</v>
+          </cell>
+          <cell r="C7" t="str">
+            <v>1405/05/05</v>
+          </cell>
+          <cell r="D7" t="str">
+            <v>1405/08/05</v>
+          </cell>
+          <cell r="E7">
+            <v>135000000</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="A8" t="str">
+            <v>DR Ata Heydari</v>
+          </cell>
+          <cell r="B8" t="str">
+            <v>Naser</v>
+          </cell>
+          <cell r="E8">
+            <v>150000000</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="A9" t="str">
+            <v>Dr Azhie</v>
+          </cell>
+          <cell r="B9" t="str">
+            <v>Naser</v>
+          </cell>
+          <cell r="C9" t="str">
+            <v>1405/05/19</v>
+          </cell>
+          <cell r="D9" t="str">
+            <v>1405/08/19</v>
+          </cell>
+          <cell r="E9">
+            <v>140000000</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="A10" t="str">
+            <v>Dr Azadeh MirMaasoumi</v>
+          </cell>
+          <cell r="B10" t="str">
+            <v>Sara</v>
+          </cell>
+          <cell r="C10" t="str">
+            <v>1405/03/16</v>
+          </cell>
+          <cell r="D10" t="str">
+            <v>1405/05/16</v>
+          </cell>
+          <cell r="E10">
+            <v>45000000</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="A11" t="str">
+            <v>Dr Homa Sharifi</v>
+          </cell>
+          <cell r="B11" t="str">
+            <v>Sara</v>
+          </cell>
+          <cell r="C11" t="str">
+            <v>1405/04/08</v>
+          </cell>
+          <cell r="D11" t="str">
+            <v>1405/07/08</v>
+          </cell>
+          <cell r="E11">
+            <v>27000000</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="A12" t="str">
+            <v>Dr Zarin BadiNi</v>
+          </cell>
+          <cell r="B12" t="str">
+            <v>Sanam</v>
+          </cell>
+          <cell r="C12" t="str">
+            <v>1405/04/29</v>
+          </cell>
+          <cell r="D12" t="str">
+            <v>1405/07/29</v>
+          </cell>
+          <cell r="E12">
+            <v>240000000</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="A13" t="str">
+            <v>DR Zeynab Tavana</v>
+          </cell>
+          <cell r="B13" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C13" t="str">
+            <v>1405/05/19</v>
+          </cell>
+          <cell r="D13" t="str">
+            <v>1405/08/19</v>
+          </cell>
+          <cell r="E13">
+            <v>8800000</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="A14" t="str">
+            <v>Dr. Farshad Sadeghi</v>
+          </cell>
+          <cell r="B14" t="str">
+            <v>Sara</v>
+          </cell>
+          <cell r="C14" t="str">
+            <v>1405/04/10</v>
+          </cell>
+          <cell r="D14" t="str">
+            <v>1405/07/10</v>
+          </cell>
+          <cell r="E14">
+            <v>60000000</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="A15" t="str">
+            <v>Dr. Amir Bastani</v>
+          </cell>
+          <cell r="B15" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C15" t="str">
+            <v>1405/03/09</v>
+          </cell>
+          <cell r="D15" t="str">
+            <v>1405/06/09</v>
+          </cell>
+          <cell r="E15">
+            <v>36000000</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="A16" t="str">
+            <v>Dr. Ghazi</v>
+          </cell>
+          <cell r="B16" t="str">
+            <v>Naser</v>
+          </cell>
+          <cell r="C16" t="str">
+            <v>1405/06/04</v>
+          </cell>
+          <cell r="D16" t="str">
+            <v>1405/09/04</v>
+          </cell>
+          <cell r="E16">
+            <v>427000000</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="A17" t="str">
+            <v>Dr. Hadi Mansouri</v>
+          </cell>
+          <cell r="B17" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C17" t="str">
+            <v>1405/04/02</v>
+          </cell>
+          <cell r="D17" t="str">
+            <v>1405/07/02</v>
+          </cell>
+          <cell r="E17">
+            <v>46200000</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="A18" t="str">
+            <v>Dr. Izadpanah</v>
+          </cell>
+          <cell r="B18" t="str">
+            <v>Sara</v>
+          </cell>
+          <cell r="C18" t="str">
+            <v>1405/04/28</v>
+          </cell>
+          <cell r="D18" t="str">
+            <v>1405/07/28</v>
+          </cell>
+          <cell r="E18">
+            <v>75000000</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="A19" t="str">
+            <v>Dr. Hengame Mehrfar</v>
+          </cell>
+          <cell r="B19" t="str">
+            <v>shahrzad</v>
+          </cell>
+          <cell r="C19" t="str">
+            <v>1405/05/25</v>
+          </cell>
+          <cell r="D19" t="str">
+            <v>1405/08/25</v>
+          </cell>
+          <cell r="E19">
+            <v>46200000</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="A20" t="str">
+            <v>Dr. Mohammad Borzoyi</v>
+          </cell>
+          <cell r="B20" t="str">
+            <v>shahrzad</v>
+          </cell>
+          <cell r="C20" t="str">
+            <v>1405/03/04</v>
+          </cell>
+          <cell r="D20" t="str">
+            <v>1405/06/04</v>
+          </cell>
+          <cell r="E20">
+            <v>49500000</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="A21" t="str">
+            <v>Dr. Mayryam Farokhshahi</v>
+          </cell>
+          <cell r="B21" t="str">
+            <v>shahrzad</v>
+          </cell>
+          <cell r="C21" t="str">
+            <v>1405/06/02</v>
+          </cell>
+          <cell r="D21" t="str">
+            <v>1405/09/02</v>
+          </cell>
+          <cell r="E21">
+            <v>6600000</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="A22" t="str">
+            <v>Dr. Kartalayi</v>
+          </cell>
+          <cell r="B22" t="str">
+            <v>shahrzad</v>
+          </cell>
+          <cell r="C22" t="str">
+            <v>1405/05/29</v>
+          </cell>
+          <cell r="D22" t="str">
+            <v>1405/08/29</v>
+          </cell>
+          <cell r="E22">
+            <v>41580000</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="A23" t="str">
+            <v>Dr. Negin Asna Asahari</v>
+          </cell>
+          <cell r="B23" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C23" t="str">
+            <v>1405/06/16</v>
+          </cell>
+          <cell r="D23" t="str">
+            <v>1405/09/16</v>
+          </cell>
+          <cell r="E23">
+            <v>23100000</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="A24" t="str">
+            <v>Dr. Natami</v>
+          </cell>
+          <cell r="B24" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C24" t="str">
+            <v>1405/03/25</v>
+          </cell>
+          <cell r="D24" t="str">
+            <v>1405/06/25</v>
+          </cell>
+          <cell r="E24">
+            <v>33000000</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="A25" t="str">
+            <v>Dr. YazdanShenas</v>
+          </cell>
+          <cell r="B25" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C25" t="str">
+            <v>1405/03/17</v>
+          </cell>
+          <cell r="D25" t="str">
+            <v>1405/06/17</v>
+          </cell>
+          <cell r="E25">
+            <v>170000000</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="A26" t="str">
+            <v>Dr. Sahar Tavakoli</v>
+          </cell>
+          <cell r="B26" t="str">
+            <v>shahrzad</v>
+          </cell>
+          <cell r="C26" t="str">
+            <v>1405/06/16</v>
+          </cell>
+          <cell r="D26" t="str">
+            <v>1405/09/16</v>
+          </cell>
+          <cell r="E26">
+            <v>30000000</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="A27" t="str">
+            <v>Farzin Khorvash</v>
+          </cell>
+          <cell r="B27" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C27" t="str">
+            <v>1405/04/04</v>
+          </cell>
+          <cell r="D27" t="str">
+            <v>1405/07/04</v>
+          </cell>
+          <cell r="E27">
+            <v>49500000</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="A28" t="str">
+            <v>Farzane Mortazavi Far</v>
+          </cell>
+          <cell r="B28" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C28" t="str">
+            <v>1405/04/27</v>
+          </cell>
+          <cell r="D28" t="str">
+            <v>1405/07/27</v>
+          </cell>
+          <cell r="E28">
+            <v>72600000</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="A29" t="str">
+            <v>Farnaz Bagherian</v>
+          </cell>
+          <cell r="B29" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C29" t="str">
+            <v>1405/05/24</v>
+          </cell>
+          <cell r="D29" t="str">
+            <v>1405/08/24</v>
+          </cell>
+          <cell r="E29">
+            <v>6600000</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="A30" t="str">
+            <v>Hamed Mahmoudi</v>
+          </cell>
+          <cell r="B30" t="str">
+            <v>Naser</v>
+          </cell>
+          <cell r="C30" t="str">
+            <v>1405/05/06</v>
+          </cell>
+          <cell r="D30" t="str">
+            <v>1405/08/06</v>
+          </cell>
+          <cell r="E30">
+            <v>206000000</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="A31" t="str">
+            <v>Fateme Golestani</v>
+          </cell>
+          <cell r="B31" t="str">
+            <v>Sara</v>
+          </cell>
+          <cell r="C31" t="str">
+            <v>1405/03/30</v>
+          </cell>
+          <cell r="D31" t="str">
+            <v>1405/06/30</v>
+          </cell>
+          <cell r="E31">
+            <v>34000000</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="A32" t="str">
+            <v>HamidReza Ziayie</v>
+          </cell>
+          <cell r="B32" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C32" t="str">
+            <v>1405/03/18</v>
+          </cell>
+          <cell r="D32" t="str">
+            <v>1405/06/18</v>
+          </cell>
+          <cell r="E32">
+            <v>76000000</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="A33" t="str">
+            <v>Hamid MehraBi</v>
+          </cell>
+          <cell r="B33" t="str">
+            <v>Mohamad</v>
+          </cell>
+          <cell r="C33" t="str">
+            <v>1405/04/16</v>
+          </cell>
+          <cell r="D33" t="str">
+            <v>1405/07/16</v>
+          </cell>
+          <cell r="E33">
+            <v>60000000</v>
+          </cell>
+        </row>
+        <row r="34">
+          <cell r="A34" t="str">
+            <v>HonarVAr</v>
+          </cell>
+          <cell r="B34" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C34" t="str">
+            <v>1405/02/30</v>
+          </cell>
+          <cell r="D34" t="str">
+            <v>1405/05/30</v>
+          </cell>
+          <cell r="E34">
+            <v>39600000</v>
+          </cell>
+        </row>
+        <row r="35">
+          <cell r="A35" t="str">
+            <v>Hashem Rafie Zadeh</v>
+          </cell>
+          <cell r="B35" t="str">
+            <v>Mohamad</v>
+          </cell>
+          <cell r="C35" t="str">
+            <v>1405/04/20</v>
+          </cell>
+          <cell r="D35" t="str">
+            <v>1405/07/20</v>
+          </cell>
+          <cell r="E35">
+            <v>42900000</v>
+          </cell>
+        </row>
+        <row r="36">
+          <cell r="A36" t="str">
+            <v>Keyvan Rezaie</v>
+          </cell>
+          <cell r="B36" t="str">
+            <v>Naser</v>
+          </cell>
+          <cell r="C36" t="str">
+            <v>1405/05/26</v>
+          </cell>
+          <cell r="D36" t="str">
+            <v>1405/08/26</v>
+          </cell>
+          <cell r="E36">
+            <v>99000000</v>
+          </cell>
+        </row>
+        <row r="37">
+          <cell r="A37" t="str">
+            <v>Khashayar KhaniZadeh</v>
+          </cell>
+          <cell r="B37" t="str">
+            <v>Naser</v>
+          </cell>
+          <cell r="C37" t="str">
+            <v>1405/05/11</v>
+          </cell>
+          <cell r="D37" t="str">
+            <v>1405/08/11</v>
+          </cell>
+          <cell r="E37">
+            <v>44000000</v>
+          </cell>
+        </row>
+        <row r="38">
+          <cell r="A38" t="str">
+            <v>Lale Izadi</v>
+          </cell>
+          <cell r="B38" t="str">
+            <v>Sanam</v>
+          </cell>
+          <cell r="C38" t="str">
+            <v>1405/05/06</v>
+          </cell>
+          <cell r="D38" t="str">
+            <v>1405/08/06</v>
+          </cell>
+          <cell r="E38">
+            <v>80000000</v>
+          </cell>
+        </row>
+        <row r="39">
+          <cell r="A39" t="str">
+            <v>KIMIA Ghasemi</v>
+          </cell>
+          <cell r="B39" t="str">
+            <v>Mohamad</v>
+          </cell>
+          <cell r="C39" t="str">
+            <v>1405/05/03</v>
+          </cell>
+          <cell r="D39" t="str">
+            <v>1405/08/03</v>
+          </cell>
+          <cell r="E39">
+            <v>29700000</v>
+          </cell>
+        </row>
+        <row r="40">
+          <cell r="A40" t="str">
+            <v>Khatereh Jafari</v>
+          </cell>
+          <cell r="B40" t="str">
+            <v>Sanam</v>
+          </cell>
+          <cell r="C40" t="str">
+            <v>1405/04/08</v>
+          </cell>
+          <cell r="D40" t="str">
+            <v>1405/07/08</v>
+          </cell>
+          <cell r="E40">
+            <v>30000000</v>
+          </cell>
+        </row>
+        <row r="41">
+          <cell r="A41" t="str">
+            <v>Mansoureh AmirShahi</v>
+          </cell>
+          <cell r="B41" t="str">
+            <v>Nastaran</v>
+          </cell>
+          <cell r="C41" t="str">
+            <v>1405/06/16</v>
+          </cell>
+          <cell r="D41" t="str">
+            <v>1405/09/16</v>
+          </cell>
+          <cell r="E41">
+            <v>33000000</v>
+          </cell>
+        </row>
+        <row r="42">
+          <cell r="A42" t="str">
+            <v>Maasoume Zare</v>
+          </cell>
+          <cell r="B42" t="str">
+            <v>Shaqayeq</v>
+          </cell>
+          <cell r="C42" t="str">
+            <v>1405/04/28</v>
+          </cell>
+          <cell r="D42" t="str">
+            <v>1405/07/28</v>
+          </cell>
+          <cell r="E42">
+            <v>30000000</v>
+          </cell>
+        </row>
+        <row r="43">
+          <cell r="A43" t="str">
+            <v>Maryam Gholami</v>
+          </cell>
+          <cell r="B43" t="str">
+            <v>Mohamad</v>
+          </cell>
+          <cell r="C43" t="str">
+            <v>1405/02/16</v>
+          </cell>
+          <cell r="D43" t="str">
+            <v>1405/05/16</v>
+          </cell>
+          <cell r="E43">
+            <v>46200000</v>
+          </cell>
+        </row>
+        <row r="44">
+          <cell r="A44" t="str">
+            <v>Maryam DadKhah</v>
+          </cell>
+          <cell r="B44" t="str">
+            <v>Sanam</v>
+          </cell>
+          <cell r="C44" t="str">
+            <v>1405/05/27</v>
+          </cell>
+          <cell r="D44" t="str">
+            <v>1405/08/27</v>
+          </cell>
+          <cell r="E44">
+            <v>40000000</v>
+          </cell>
+        </row>
+        <row r="45">
+          <cell r="A45" t="str">
+            <v>Meysam Ghanbari</v>
+          </cell>
+          <cell r="B45" t="str">
+            <v>shahrzad</v>
+          </cell>
+          <cell r="C45" t="str">
+            <v>1405/05/28</v>
+          </cell>
+          <cell r="D45" t="str">
+            <v>1405/08/28</v>
+          </cell>
+          <cell r="E45">
+            <v>82500000</v>
+          </cell>
+        </row>
+        <row r="46">
+          <cell r="A46" t="str">
+            <v>Mazaher Hadi</v>
+          </cell>
+          <cell r="B46" t="str">
+            <v>shahrzad</v>
+          </cell>
+          <cell r="C46" t="str">
+            <v>1405/05/10</v>
+          </cell>
+          <cell r="D46" t="str">
+            <v>1405/08/10</v>
+          </cell>
+          <cell r="E46">
+            <v>58000000</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4544,8 +5351,13 @@
       <c r="F32" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="G32" s="1"/>
-      <c r="H32" s="12"/>
+      <c r="G32" s="55" t="s">
+        <v>26</v>
+      </c>
+      <c r="H32" s="12">
+        <f>VLOOKUP(A32,[1]Sheet2!A:E,5,0)</f>
+        <v>132000000</v>
+      </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
@@ -4566,8 +5378,13 @@
       <c r="F33" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="G33" s="1"/>
-      <c r="H33" s="12"/>
+      <c r="G33" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H33" s="12">
+        <f>VLOOKUP(A33,[1]Sheet2!A:E,5,0)</f>
+        <v>132000000</v>
+      </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
@@ -4588,8 +5405,13 @@
       <c r="F34" s="24" t="s">
         <v>188</v>
       </c>
-      <c r="G34" s="1"/>
-      <c r="H34" s="12"/>
+      <c r="G34" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" s="12">
+        <f>VLOOKUP(A34,[1]Sheet2!A:E,5,0)</f>
+        <v>55000000</v>
+      </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -4610,8 +5432,14 @@
       <c r="F35" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="G35" s="1"/>
-      <c r="H35" s="12"/>
+      <c r="G35" s="1" t="str">
+        <f>VLOOKUP(A35,[1]Sheet2!A:B,2,0)</f>
+        <v>Sanam</v>
+      </c>
+      <c r="H35" s="12">
+        <f>VLOOKUP(A35,[1]Sheet2!A:E,5,0)</f>
+        <v>30600000</v>
+      </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -4654,8 +5482,14 @@
       <c r="F37" s="26" t="s">
         <v>199</v>
       </c>
-      <c r="G37" s="1"/>
-      <c r="H37" s="12"/>
+      <c r="G37" s="1" t="str">
+        <f>VLOOKUP(A37,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H37" s="12">
+        <f>VLOOKUP(A37,[1]Sheet2!A:E,5,0)</f>
+        <v>20000000</v>
+      </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -4676,8 +5510,14 @@
       <c r="F38" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="G38" s="1"/>
-      <c r="H38" s="12"/>
+      <c r="G38" s="1" t="str">
+        <f>VLOOKUP(A38,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H38" s="12">
+        <f>VLOOKUP(A38,[1]Sheet2!A:E,5,0)</f>
+        <v>150000000</v>
+      </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
@@ -4698,8 +5538,14 @@
       <c r="F39" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="G39" s="1"/>
-      <c r="H39" s="12"/>
+      <c r="G39" s="1" t="str">
+        <f>VLOOKUP(A39,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H39" s="12">
+        <f>VLOOKUP(A39,[1]Sheet2!A:E,5,0)</f>
+        <v>135000000</v>
+      </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -4720,8 +5566,14 @@
       <c r="F40" s="27" t="s">
         <v>222</v>
       </c>
-      <c r="G40" s="1"/>
-      <c r="H40" s="12"/>
+      <c r="G40" s="1" t="str">
+        <f>VLOOKUP(A40,[1]Sheet2!A:B,2,0)</f>
+        <v>Sanam</v>
+      </c>
+      <c r="H40" s="12">
+        <f>VLOOKUP(A40,[1]Sheet2!A:E,5,0)</f>
+        <v>60000000</v>
+      </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -4742,8 +5594,14 @@
       <c r="F41" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="G41" s="1"/>
-      <c r="H41" s="12"/>
+      <c r="G41" s="1" t="str">
+        <f>VLOOKUP(A41,[1]Sheet2!A:B,2,0)</f>
+        <v>Sara</v>
+      </c>
+      <c r="H41" s="12">
+        <f>VLOOKUP(A41,[1]Sheet2!A:E,5,0)</f>
+        <v>45000000</v>
+      </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
@@ -4764,8 +5622,14 @@
       <c r="F42" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="G42" s="1"/>
-      <c r="H42" s="12"/>
+      <c r="G42" s="1" t="str">
+        <f>VLOOKUP(A42,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H42" s="12">
+        <f>VLOOKUP(A42,[1]Sheet2!A:E,5,0)</f>
+        <v>140000000</v>
+      </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
@@ -4852,8 +5716,14 @@
       <c r="F46" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="G46" s="1"/>
-      <c r="H46" s="12"/>
+      <c r="G46" s="1" t="str">
+        <f>VLOOKUP(A46,[1]Sheet2!A:B,2,0)</f>
+        <v>Sara</v>
+      </c>
+      <c r="H46" s="12">
+        <f>VLOOKUP(A46,[1]Sheet2!A:E,5,0)</f>
+        <v>27000000</v>
+      </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
@@ -5204,8 +6074,14 @@
       <c r="F62" s="34" t="s">
         <v>326</v>
       </c>
-      <c r="G62" s="1"/>
-      <c r="H62" s="12"/>
+      <c r="G62" s="1" t="str">
+        <f>VLOOKUP(A62,[1]Sheet2!A:B,2,0)</f>
+        <v>Sanam</v>
+      </c>
+      <c r="H62" s="12">
+        <f>VLOOKUP(A62,[1]Sheet2!A:E,5,0)</f>
+        <v>240000000</v>
+      </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
@@ -5226,8 +6102,14 @@
       <c r="F63" s="34" t="s">
         <v>326</v>
       </c>
-      <c r="G63" s="1"/>
-      <c r="H63" s="12"/>
+      <c r="G63" s="1" t="str">
+        <f>VLOOKUP(A63,[1]Sheet2!A:B,2,0)</f>
+        <v>Sanam</v>
+      </c>
+      <c r="H63" s="12">
+        <f>VLOOKUP(A63,[1]Sheet2!A:E,5,0)</f>
+        <v>240000000</v>
+      </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
@@ -5248,8 +6130,14 @@
       <c r="F64" s="34" t="s">
         <v>326</v>
       </c>
-      <c r="G64" s="1"/>
-      <c r="H64" s="12"/>
+      <c r="G64" s="1" t="str">
+        <f>VLOOKUP(A64,[1]Sheet2!A:B,2,0)</f>
+        <v>Sanam</v>
+      </c>
+      <c r="H64" s="12">
+        <f>VLOOKUP(A64,[1]Sheet2!A:E,5,0)</f>
+        <v>240000000</v>
+      </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
@@ -5270,8 +6158,14 @@
       <c r="F65" s="34" t="s">
         <v>326</v>
       </c>
-      <c r="G65" s="1"/>
-      <c r="H65" s="12"/>
+      <c r="G65" s="1" t="str">
+        <f>VLOOKUP(A65,[1]Sheet2!A:B,2,0)</f>
+        <v>Sanam</v>
+      </c>
+      <c r="H65" s="12">
+        <f>VLOOKUP(A65,[1]Sheet2!A:E,5,0)</f>
+        <v>240000000</v>
+      </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
@@ -5292,8 +6186,14 @@
       <c r="F66" s="34" t="s">
         <v>326</v>
       </c>
-      <c r="G66" s="1"/>
-      <c r="H66" s="12"/>
+      <c r="G66" s="1" t="str">
+        <f>VLOOKUP(A66,[1]Sheet2!A:B,2,0)</f>
+        <v>Sanam</v>
+      </c>
+      <c r="H66" s="12">
+        <f>VLOOKUP(A66,[1]Sheet2!A:E,5,0)</f>
+        <v>240000000</v>
+      </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
@@ -5314,8 +6214,14 @@
       <c r="F67" s="35" t="s">
         <v>344</v>
       </c>
-      <c r="G67" s="1"/>
-      <c r="H67" s="12"/>
+      <c r="G67" s="1" t="str">
+        <f>VLOOKUP(A67,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H67" s="12">
+        <f>VLOOKUP(A67,[1]Sheet2!A:E,5,0)</f>
+        <v>8800000</v>
+      </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
@@ -5336,8 +6242,14 @@
       <c r="F68" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="G68" s="1"/>
-      <c r="H68" s="12"/>
+      <c r="G68" s="1" t="str">
+        <f>VLOOKUP(A68,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H68" s="12">
+        <f>VLOOKUP(A68,[1]Sheet2!A:E,5,0)</f>
+        <v>36000000</v>
+      </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
@@ -5380,8 +6292,14 @@
       <c r="F70" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="G70" s="1"/>
-      <c r="H70" s="12"/>
+      <c r="G70" s="1" t="str">
+        <f>VLOOKUP(A70,[1]Sheet2!A:B,2,0)</f>
+        <v>Sara</v>
+      </c>
+      <c r="H70" s="12">
+        <f>VLOOKUP(A70,[1]Sheet2!A:E,5,0)</f>
+        <v>60000000</v>
+      </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
@@ -5402,8 +6320,14 @@
       <c r="F71" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="G71" s="1"/>
-      <c r="H71" s="12"/>
+      <c r="G71" s="1" t="str">
+        <f>VLOOKUP(A71,[1]Sheet2!A:B,2,0)</f>
+        <v>Sara</v>
+      </c>
+      <c r="H71" s="12">
+        <f>VLOOKUP(A71,[1]Sheet2!A:E,5,0)</f>
+        <v>60000000</v>
+      </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
@@ -5424,8 +6348,14 @@
       <c r="F72" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="G72" s="1"/>
-      <c r="H72" s="12"/>
+      <c r="G72" s="1" t="str">
+        <f>VLOOKUP(A72,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H72" s="12">
+        <f>VLOOKUP(A72,[1]Sheet2!A:E,5,0)</f>
+        <v>427000000</v>
+      </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
@@ -5446,8 +6376,14 @@
       <c r="F73" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="G73" s="1"/>
-      <c r="H73" s="12"/>
+      <c r="G73" s="1" t="str">
+        <f>VLOOKUP(A73,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H73" s="12">
+        <f>VLOOKUP(A73,[1]Sheet2!A:E,5,0)</f>
+        <v>427000000</v>
+      </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
@@ -5468,8 +6404,14 @@
       <c r="F74" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="G74" s="1"/>
-      <c r="H74" s="12"/>
+      <c r="G74" s="1" t="str">
+        <f>VLOOKUP(A74,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H74" s="12">
+        <f>VLOOKUP(A74,[1]Sheet2!A:E,5,0)</f>
+        <v>427000000</v>
+      </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
@@ -5490,8 +6432,14 @@
       <c r="F75" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="G75" s="1"/>
-      <c r="H75" s="12"/>
+      <c r="G75" s="1" t="str">
+        <f>VLOOKUP(A75,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H75" s="12">
+        <f>VLOOKUP(A75,[1]Sheet2!A:E,5,0)</f>
+        <v>46200000</v>
+      </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
@@ -5512,8 +6460,14 @@
       <c r="F76" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="G76" s="1"/>
-      <c r="H76" s="12"/>
+      <c r="G76" s="1" t="str">
+        <f>VLOOKUP(A76,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H76" s="12">
+        <f>VLOOKUP(A76,[1]Sheet2!A:E,5,0)</f>
+        <v>46200000</v>
+      </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
@@ -5534,8 +6488,13 @@
       <c r="F77" s="6" t="s">
         <v>388</v>
       </c>
-      <c r="G77" s="1"/>
-      <c r="H77" s="12"/>
+      <c r="G77" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H77" s="12">
+        <f>VLOOKUP(A77,[1]Sheet2!A:E,5,0)</f>
+        <v>46200000</v>
+      </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
@@ -5556,8 +6515,14 @@
       <c r="F78" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="G78" s="1"/>
-      <c r="H78" s="12"/>
+      <c r="G78" s="1" t="str">
+        <f>VLOOKUP(A78,[1]Sheet2!A:B,2,0)</f>
+        <v>Sara</v>
+      </c>
+      <c r="H78" s="12">
+        <f>VLOOKUP(A78,[1]Sheet2!A:E,5,0)</f>
+        <v>75000000</v>
+      </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
@@ -5578,8 +6543,14 @@
       <c r="F79" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="G79" s="1"/>
-      <c r="H79" s="12"/>
+      <c r="G79" s="1" t="str">
+        <f>VLOOKUP(A79,[1]Sheet2!A:B,2,0)</f>
+        <v>Sara</v>
+      </c>
+      <c r="H79" s="12">
+        <f>VLOOKUP(A79,[1]Sheet2!A:E,5,0)</f>
+        <v>75000000</v>
+      </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
@@ -5600,8 +6571,13 @@
       <c r="F80" s="6" t="s">
         <v>400</v>
       </c>
-      <c r="G80" s="1"/>
-      <c r="H80" s="12"/>
+      <c r="G80" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H80" s="12">
+        <f>VLOOKUP(A80,[1]Sheet2!A:E,5,0)</f>
+        <v>41580000</v>
+      </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
@@ -5622,8 +6598,13 @@
       <c r="F81" s="6" t="s">
         <v>406</v>
       </c>
-      <c r="G81" s="1"/>
-      <c r="H81" s="12"/>
+      <c r="G81" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H81" s="12">
+        <f>VLOOKUP(A81,[1]Sheet2!A:E,5,0)</f>
+        <v>6600000</v>
+      </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
@@ -5644,8 +6625,13 @@
       <c r="F82" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="G82" s="1"/>
-      <c r="H82" s="12"/>
+      <c r="G82" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H82" s="12">
+        <f>VLOOKUP(A82,[1]Sheet2!A:E,5,0)</f>
+        <v>49500000</v>
+      </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
@@ -5666,8 +6652,14 @@
       <c r="F83" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="G83" s="1"/>
-      <c r="H83" s="12"/>
+      <c r="G83" s="1" t="str">
+        <f>VLOOKUP(A83,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H83" s="12">
+        <f>VLOOKUP(A83,[1]Sheet2!A:E,5,0)</f>
+        <v>33000000</v>
+      </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
@@ -5688,8 +6680,14 @@
       <c r="F84" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="G84" s="1"/>
-      <c r="H84" s="12"/>
+      <c r="G84" s="1" t="str">
+        <f>VLOOKUP(A84,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H84" s="12">
+        <f>VLOOKUP(A84,[1]Sheet2!A:E,5,0)</f>
+        <v>23100000</v>
+      </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
@@ -5710,8 +6708,14 @@
       <c r="F85" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="G85" s="1"/>
-      <c r="H85" s="12"/>
+      <c r="G85" s="1" t="str">
+        <f>VLOOKUP(A85,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H85" s="12">
+        <f>VLOOKUP(A85,[1]Sheet2!A:E,5,0)</f>
+        <v>23100000</v>
+      </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
@@ -5732,8 +6736,13 @@
       <c r="F86" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="G86" s="1"/>
-      <c r="H86" s="12"/>
+      <c r="G86" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H86" s="12">
+        <f>VLOOKUP(A86,[1]Sheet2!A:E,5,0)</f>
+        <v>30000000</v>
+      </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
@@ -5776,8 +6785,14 @@
       <c r="F88" s="6" t="s">
         <v>445</v>
       </c>
-      <c r="G88" s="1"/>
-      <c r="H88" s="12"/>
+      <c r="G88" s="1" t="str">
+        <f>VLOOKUP(A88,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H88" s="12">
+        <f>VLOOKUP(A88,[1]Sheet2!A:E,5,0)</f>
+        <v>170000000</v>
+      </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
@@ -5798,8 +6813,14 @@
       <c r="F89" s="6" t="s">
         <v>445</v>
       </c>
-      <c r="G89" s="1"/>
-      <c r="H89" s="12"/>
+      <c r="G89" s="1" t="str">
+        <f>VLOOKUP(A89,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H89" s="12">
+        <f>VLOOKUP(A89,[1]Sheet2!A:E,5,0)</f>
+        <v>170000000</v>
+      </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
@@ -5864,8 +6885,14 @@
       <c r="F92" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G92" s="1"/>
-      <c r="H92" s="12"/>
+      <c r="G92" s="1" t="str">
+        <f>VLOOKUP(A92,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H92" s="12">
+        <f>VLOOKUP(A92,[1]Sheet2!A:E,5,0)</f>
+        <v>6600000</v>
+      </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
@@ -5886,8 +6913,14 @@
       <c r="F93" s="6" t="s">
         <v>467</v>
       </c>
-      <c r="G93" s="1"/>
-      <c r="H93" s="12"/>
+      <c r="G93" s="1" t="str">
+        <f>VLOOKUP(A93,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H93" s="12">
+        <f>VLOOKUP(A93,[1]Sheet2!A:E,5,0)</f>
+        <v>72600000</v>
+      </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
@@ -5908,8 +6941,14 @@
       <c r="F94" s="36" t="s">
         <v>472</v>
       </c>
-      <c r="G94" s="1"/>
-      <c r="H94" s="12"/>
+      <c r="G94" s="1" t="str">
+        <f>VLOOKUP(A94,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H94" s="12">
+        <f>VLOOKUP(A94,[1]Sheet2!A:E,5,0)</f>
+        <v>49500000</v>
+      </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
@@ -5930,8 +6969,14 @@
       <c r="F95" s="28" t="s">
         <v>255</v>
       </c>
-      <c r="G95" s="1"/>
-      <c r="H95" s="12"/>
+      <c r="G95" s="1" t="str">
+        <f>VLOOKUP(A95,[1]Sheet2!A:B,2,0)</f>
+        <v>Sara</v>
+      </c>
+      <c r="H95" s="12">
+        <f>VLOOKUP(A95,[1]Sheet2!A:E,5,0)</f>
+        <v>34000000</v>
+      </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
@@ -5974,8 +7019,14 @@
       <c r="F97" s="6" t="s">
         <v>487</v>
       </c>
-      <c r="G97" s="1"/>
-      <c r="H97" s="12"/>
+      <c r="G97" s="1" t="str">
+        <f>VLOOKUP(A97,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H97" s="12">
+        <f>VLOOKUP(A97,[1]Sheet2!A:E,5,0)</f>
+        <v>206000000</v>
+      </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
@@ -5996,8 +7047,14 @@
       <c r="F98" s="6" t="s">
         <v>487</v>
       </c>
-      <c r="G98" s="1"/>
-      <c r="H98" s="12"/>
+      <c r="G98" s="1" t="str">
+        <f>VLOOKUP(A98,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H98" s="12">
+        <f>VLOOKUP(A98,[1]Sheet2!A:E,5,0)</f>
+        <v>206000000</v>
+      </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
@@ -6018,8 +7075,13 @@
       <c r="F99" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="G99" s="1"/>
-      <c r="H99" s="12"/>
+      <c r="G99" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H99" s="12">
+        <f>VLOOKUP(A99,[1]Sheet2!A:E,5,0)</f>
+        <v>60000000</v>
+      </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
@@ -6040,8 +7102,14 @@
       <c r="F100" s="37" t="s">
         <v>500</v>
       </c>
-      <c r="G100" s="1"/>
-      <c r="H100" s="12"/>
+      <c r="G100" s="1" t="str">
+        <f>VLOOKUP(A100,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H100" s="12">
+        <f>VLOOKUP(A100,[1]Sheet2!A:E,5,0)</f>
+        <v>76000000</v>
+      </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
@@ -6062,8 +7130,13 @@
       <c r="F101" s="38" t="s">
         <v>505</v>
       </c>
-      <c r="G101" s="1"/>
-      <c r="H101" s="12"/>
+      <c r="G101" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H101" s="12">
+        <f>VLOOKUP(A101,[1]Sheet2!A:E,5,0)</f>
+        <v>42900000</v>
+      </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
@@ -6084,8 +7157,14 @@
       <c r="F102" s="6" t="s">
         <v>511</v>
       </c>
-      <c r="G102" s="1"/>
-      <c r="H102" s="12"/>
+      <c r="G102" s="1" t="str">
+        <f>VLOOKUP(A102,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H102" s="12">
+        <f>VLOOKUP(A102,[1]Sheet2!A:E,5,0)</f>
+        <v>39600000</v>
+      </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
@@ -6370,8 +7449,14 @@
       <c r="F115" s="6" t="s">
         <v>510</v>
       </c>
-      <c r="G115" s="1"/>
-      <c r="H115" s="12"/>
+      <c r="G115" s="1" t="str">
+        <f>VLOOKUP(A115,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H115" s="12">
+        <f>VLOOKUP(A115,[1]Sheet2!A:E,5,0)</f>
+        <v>99000000</v>
+      </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
@@ -6392,8 +7477,14 @@
       <c r="F116" s="6" t="s">
         <v>510</v>
       </c>
-      <c r="G116" s="1"/>
-      <c r="H116" s="12"/>
+      <c r="G116" s="1" t="str">
+        <f>VLOOKUP(A116,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H116" s="12">
+        <f>VLOOKUP(A116,[1]Sheet2!A:E,5,0)</f>
+        <v>99000000</v>
+      </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
@@ -6414,8 +7505,14 @@
       <c r="F117" s="6" t="s">
         <v>510</v>
       </c>
-      <c r="G117" s="1"/>
-      <c r="H117" s="12"/>
+      <c r="G117" s="1" t="str">
+        <f>VLOOKUP(A117,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H117" s="12">
+        <f>VLOOKUP(A117,[1]Sheet2!A:E,5,0)</f>
+        <v>99000000</v>
+      </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
@@ -6436,8 +7533,14 @@
       <c r="F118" s="13" t="s">
         <v>571</v>
       </c>
-      <c r="G118" s="1"/>
-      <c r="H118" s="12"/>
+      <c r="G118" s="1" t="str">
+        <f>VLOOKUP(A118,[1]Sheet2!A:B,2,0)</f>
+        <v>Naser</v>
+      </c>
+      <c r="H118" s="12">
+        <f>VLOOKUP(A118,[1]Sheet2!A:E,5,0)</f>
+        <v>44000000</v>
+      </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
@@ -6458,8 +7561,14 @@
       <c r="F119" s="6" t="s">
         <v>576</v>
       </c>
-      <c r="G119" s="1"/>
-      <c r="H119" s="12"/>
+      <c r="G119" s="1" t="str">
+        <f>VLOOKUP(A119,[1]Sheet2!A:B,2,0)</f>
+        <v>Sanam</v>
+      </c>
+      <c r="H119" s="12">
+        <f>VLOOKUP(A119,[1]Sheet2!A:E,5,0)</f>
+        <v>30000000</v>
+      </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
@@ -6480,8 +7589,13 @@
       <c r="F120" s="6" t="s">
         <v>582</v>
       </c>
-      <c r="G120" s="1"/>
-      <c r="H120" s="12"/>
+      <c r="G120" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H120" s="12">
+        <f>VLOOKUP(A120,[1]Sheet2!A:E,5,0)</f>
+        <v>29700000</v>
+      </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
@@ -6502,8 +7616,14 @@
       <c r="F121" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="G121" s="1"/>
-      <c r="H121" s="12"/>
+      <c r="G121" s="1" t="str">
+        <f>VLOOKUP(A121,[1]Sheet2!A:B,2,0)</f>
+        <v>Sanam</v>
+      </c>
+      <c r="H121" s="12">
+        <f>VLOOKUP(A121,[1]Sheet2!A:E,5,0)</f>
+        <v>80000000</v>
+      </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
@@ -6524,8 +7644,13 @@
       <c r="F122" s="41" t="s">
         <v>591</v>
       </c>
-      <c r="G122" s="1"/>
-      <c r="H122" s="12"/>
+      <c r="G122" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H122" s="12">
+        <f>VLOOKUP(A122,[1]Sheet2!A:E,5,0)</f>
+        <v>30000000</v>
+      </c>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
@@ -6568,8 +7693,14 @@
       <c r="F124" s="32" t="s">
         <v>304</v>
       </c>
-      <c r="G124" s="1"/>
-      <c r="H124" s="12"/>
+      <c r="G124" s="1" t="str">
+        <f>VLOOKUP(A124,[1]Sheet2!A:B,2,0)</f>
+        <v>Nastaran</v>
+      </c>
+      <c r="H124" s="12">
+        <f>VLOOKUP(A124,[1]Sheet2!A:E,5,0)</f>
+        <v>33000000</v>
+      </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
@@ -6590,8 +7721,14 @@
       <c r="F125" s="26" t="s">
         <v>199</v>
       </c>
-      <c r="G125" s="1"/>
-      <c r="H125" s="12"/>
+      <c r="G125" s="1" t="str">
+        <f>VLOOKUP(A125,[1]Sheet2!A:B,2,0)</f>
+        <v>Sanam</v>
+      </c>
+      <c r="H125" s="12">
+        <f>VLOOKUP(A125,[1]Sheet2!A:E,5,0)</f>
+        <v>40000000</v>
+      </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
@@ -6612,8 +7749,13 @@
       <c r="F126" s="6" t="s">
         <v>607</v>
       </c>
-      <c r="G126" s="1"/>
-      <c r="H126" s="12"/>
+      <c r="G126" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H126" s="12">
+        <f>VLOOKUP(A126,[1]Sheet2!A:E,5,0)</f>
+        <v>46200000</v>
+      </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
@@ -6656,8 +7798,13 @@
       <c r="F128" s="6" t="s">
         <v>618</v>
       </c>
-      <c r="G128" s="1"/>
-      <c r="H128" s="12"/>
+      <c r="G128" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H128" s="12">
+        <f>VLOOKUP(A128,[1]Sheet2!A:E,5,0)</f>
+        <v>58000000</v>
+      </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
@@ -6700,8 +7847,13 @@
       <c r="F130" s="6" t="s">
         <v>624</v>
       </c>
-      <c r="G130" s="1"/>
-      <c r="H130" s="12"/>
+      <c r="G130" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H130" s="12">
+        <f>VLOOKUP(A130,[1]Sheet2!A:E,5,0)</f>
+        <v>82500000</v>
+      </c>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
@@ -6722,8 +7874,13 @@
       <c r="F131" s="6" t="s">
         <v>624</v>
       </c>
-      <c r="G131" s="1"/>
-      <c r="H131" s="12"/>
+      <c r="G131" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H131" s="12">
+        <f>VLOOKUP(A131,[1]Sheet2!A:E,5,0)</f>
+        <v>82500000</v>
+      </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
@@ -6744,8 +7901,13 @@
       <c r="F132" s="6" t="s">
         <v>624</v>
       </c>
-      <c r="G132" s="1"/>
-      <c r="H132" s="12"/>
+      <c r="G132" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H132" s="12">
+        <f>VLOOKUP(A132,[1]Sheet2!A:E,5,0)</f>
+        <v>82500000</v>
+      </c>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">

</xml_diff>